<commit_message>
mi version de los sort con pruebas
</commit_message>
<xml_diff>
--- a/Tarea#2.xlsx
+++ b/Tarea#2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unitechn-my.sharepoint.com/personal/ema_castellanos_unitec_edu/Documents/2026/Q2 2026/analisis de algoritmos/Semana 6/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{EBE05390-39BD-48B3-B14E-C882FAC2D8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BDE7D7D-80B9-42BF-80D0-54E3F73D7BA2}"/>
+  <xr:revisionPtr revIDLastSave="209" documentId="8_{EBE05390-39BD-48B3-B14E-C882FAC2D8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B87DC15-EDB2-4388-8534-3942377A771A}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{0331FB16-A420-4772-893E-678055F07C6C}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{0331FB16-A420-4772-893E-678055F07C6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sorts De Ema" sheetId="1" r:id="rId1"/>
@@ -179,7 +179,7 @@
     <numFmt numFmtId="164" formatCode="0.00000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,12 +212,6 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -384,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -392,15 +386,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -452,9 +437,84 @@
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -464,104 +524,29 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -924,328 +909,429 @@
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="17" width="15.6640625" customWidth="1"/>
     <col min="18" max="18" width="13.88671875" customWidth="1"/>
-    <col min="19" max="19" width="15.44140625" style="13" customWidth="1"/>
+    <col min="19" max="19" width="15.44140625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="30" t="s">
+      <c r="D1" s="48"/>
+      <c r="E1" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="31"/>
-      <c r="G1" s="34" t="s">
+      <c r="F1" s="50"/>
+      <c r="G1" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="35"/>
-      <c r="I1" s="38" t="s">
+      <c r="H1" s="52"/>
+      <c r="I1" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="39"/>
-      <c r="K1" s="42" t="s">
+      <c r="J1" s="54"/>
+      <c r="K1" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="43"/>
-      <c r="M1" s="46" t="s">
+      <c r="L1" s="56"/>
+      <c r="M1" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="47"/>
-      <c r="O1" s="48" t="s">
+      <c r="N1" s="27"/>
+      <c r="O1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="52" t="s">
+      <c r="P1" s="29"/>
+      <c r="Q1" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="53"/>
-      <c r="S1" s="11" t="s">
+      <c r="R1" s="31"/>
+      <c r="S1" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="24"/>
+      <c r="A2" s="46"/>
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="27">
+      <c r="C2" s="32">
         <v>5</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="32">
+      <c r="D2" s="33"/>
+      <c r="E2" s="34">
         <v>10</v>
       </c>
-      <c r="F2" s="33"/>
+      <c r="F2" s="35"/>
       <c r="G2" s="36">
         <v>100</v>
       </c>
       <c r="H2" s="37"/>
-      <c r="I2" s="40">
+      <c r="I2" s="38">
         <v>1000</v>
       </c>
-      <c r="J2" s="41"/>
-      <c r="K2" s="44">
+      <c r="J2" s="39"/>
+      <c r="K2" s="40">
         <v>5000</v>
       </c>
-      <c r="L2" s="45"/>
-      <c r="M2" s="22">
+      <c r="L2" s="41"/>
+      <c r="M2" s="19">
         <v>10000</v>
       </c>
-      <c r="N2" s="22">
+      <c r="N2" s="19">
         <v>10000</v>
       </c>
-      <c r="O2" s="50">
+      <c r="O2" s="42">
         <v>100000</v>
       </c>
-      <c r="P2" s="51"/>
-      <c r="Q2" s="54">
+      <c r="P2" s="43"/>
+      <c r="Q2" s="44">
         <v>500000</v>
       </c>
-      <c r="R2" s="55"/>
-      <c r="S2" s="11" t="s">
+      <c r="R2" s="45"/>
+      <c r="S2" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20" t="s">
+      <c r="B3" s="25"/>
+      <c r="C3" s="11">
+        <v>0</v>
+      </c>
+      <c r="D3" s="11">
+        <v>0</v>
+      </c>
+      <c r="E3" s="12">
+        <v>0</v>
+      </c>
+      <c r="F3" s="12">
+        <v>0</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0</v>
+      </c>
+      <c r="H3" s="13">
+        <v>0</v>
+      </c>
+      <c r="I3" s="14">
+        <v>1.006</v>
+      </c>
+      <c r="J3" s="14">
+        <v>3.01</v>
+      </c>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="16">
+        <v>177.99799999999999</v>
+      </c>
+      <c r="N3" s="16">
+        <v>113.999</v>
+      </c>
+      <c r="O3" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="20" t="s">
+      <c r="P3" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="Q3" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="R3" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="S3" s="12" t="e">
+      <c r="S3" s="9">
         <f>AVERAGE(C3:R3)</f>
-        <v>#DIV/0!</v>
+        <v>29.601299999999998</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="20" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="11">
+        <v>0</v>
+      </c>
+      <c r="D4" s="11">
+        <v>0</v>
+      </c>
+      <c r="E4" s="12">
+        <v>0</v>
+      </c>
+      <c r="F4" s="12">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13">
+        <v>0</v>
+      </c>
+      <c r="H4" s="13">
+        <v>0</v>
+      </c>
+      <c r="I4" s="14">
+        <v>4.0110000000000001</v>
+      </c>
+      <c r="J4" s="14">
+        <v>5.9969999999999999</v>
+      </c>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="16">
+        <v>878.59400000000005</v>
+      </c>
+      <c r="N4" s="16">
+        <v>472.16699999999997</v>
+      </c>
+      <c r="O4" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="20" t="s">
+      <c r="P4" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="Q4" s="21" t="s">
+      <c r="Q4" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="R4" s="21" t="s">
+      <c r="R4" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="S4" s="12" t="e">
+      <c r="S4" s="9">
         <f t="shared" ref="S4:S8" si="0">AVERAGE(C4:R4)</f>
-        <v>#DIV/0!</v>
+        <v>136.07689999999999</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="20" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="11">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11">
+        <v>0</v>
+      </c>
+      <c r="E5" s="12">
+        <v>0</v>
+      </c>
+      <c r="F5" s="12">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="14">
+        <v>11.019</v>
+      </c>
+      <c r="J5" s="14">
+        <v>7.9930000000000003</v>
+      </c>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="16">
+        <v>1019.189</v>
+      </c>
+      <c r="N5" s="16">
+        <v>973.73699999999997</v>
+      </c>
+      <c r="O5" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="P5" s="20" t="s">
+      <c r="P5" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="Q5" s="21" t="s">
+      <c r="Q5" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="R5" s="21" t="s">
+      <c r="R5" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="S5" s="12" t="e">
+      <c r="S5" s="9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>201.19380000000001</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="12" t="e">
+      <c r="B6" s="25"/>
+      <c r="C6" s="11">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11">
+        <v>0</v>
+      </c>
+      <c r="E6" s="12">
+        <v>0</v>
+      </c>
+      <c r="F6" s="12">
+        <v>0</v>
+      </c>
+      <c r="G6" s="13">
+        <v>0</v>
+      </c>
+      <c r="H6" s="13">
+        <v>0</v>
+      </c>
+      <c r="I6" s="14">
+        <v>0</v>
+      </c>
+      <c r="J6" s="14">
+        <v>2.0009999999999999</v>
+      </c>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="16">
+        <v>56.994999999999997</v>
+      </c>
+      <c r="N6" s="16">
+        <v>6.992</v>
+      </c>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>6.5987999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="12" t="e">
+      <c r="B7" s="25"/>
+      <c r="C7" s="11">
+        <v>0</v>
+      </c>
+      <c r="D7" s="11">
+        <v>0</v>
+      </c>
+      <c r="E7" s="12">
+        <v>0</v>
+      </c>
+      <c r="F7" s="12">
+        <v>0</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0</v>
+      </c>
+      <c r="I7" s="14">
+        <v>0</v>
+      </c>
+      <c r="J7" s="14">
+        <v>0</v>
+      </c>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="16">
+        <v>7.9960000000000004</v>
+      </c>
+      <c r="N7" s="16">
+        <v>3.9929999999999999</v>
+      </c>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>1.1989000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="12" t="e">
+      <c r="B8" s="25"/>
+      <c r="C8" s="11">
+        <v>0</v>
+      </c>
+      <c r="D8" s="11">
+        <v>0</v>
+      </c>
+      <c r="E8" s="12">
+        <v>0</v>
+      </c>
+      <c r="F8" s="12">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="5">
+        <v>6.98</v>
+      </c>
+      <c r="N8" s="5">
+        <v>2.9980000000000002</v>
+      </c>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.99780000000000013</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29" t="s">
+      <c r="D9" s="20"/>
+      <c r="E9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29" t="s">
+      <c r="F9" s="20"/>
+      <c r="G9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29" t="s">
+      <c r="H9" s="20"/>
+      <c r="I9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="29"/>
-      <c r="K9" s="29" t="s">
+      <c r="J9" s="20"/>
+      <c r="K9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="L9" s="29"/>
-      <c r="M9" s="29" t="s">
+      <c r="L9" s="20"/>
+      <c r="M9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N9" s="29"/>
-      <c r="O9" s="29" t="s">
+      <c r="N9" s="20"/>
+      <c r="O9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="29" t="s">
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="R9" s="29"/>
+      <c r="R9" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="Q1:R1"/>
-    <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="G2:H2"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C9:D9"/>
@@ -1257,6 +1343,25 @@
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="M1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1272,466 +1377,466 @@
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="17" width="15.6640625" customWidth="1"/>
     <col min="18" max="18" width="13.88671875" customWidth="1"/>
-    <col min="19" max="19" width="18.5546875" style="13" customWidth="1"/>
+    <col min="19" max="19" width="18.5546875" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="30" t="s">
+      <c r="D1" s="48"/>
+      <c r="E1" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="31"/>
-      <c r="G1" s="34" t="s">
+      <c r="F1" s="50"/>
+      <c r="G1" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="35"/>
-      <c r="I1" s="38" t="s">
+      <c r="H1" s="52"/>
+      <c r="I1" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="39"/>
-      <c r="K1" s="42" t="s">
+      <c r="J1" s="54"/>
+      <c r="K1" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="43"/>
-      <c r="M1" s="46" t="s">
+      <c r="L1" s="56"/>
+      <c r="M1" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="47"/>
-      <c r="O1" s="48" t="s">
+      <c r="N1" s="27"/>
+      <c r="O1" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="52" t="s">
+      <c r="P1" s="29"/>
+      <c r="Q1" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="R1" s="53"/>
-      <c r="S1" s="11" t="s">
+      <c r="R1" s="31"/>
+      <c r="S1" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="24"/>
+      <c r="A2" s="46"/>
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="27">
+      <c r="C2" s="32">
         <v>5</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="32">
+      <c r="D2" s="33"/>
+      <c r="E2" s="34">
         <v>10</v>
       </c>
-      <c r="F2" s="33"/>
+      <c r="F2" s="35"/>
       <c r="G2" s="36">
         <v>100</v>
       </c>
       <c r="H2" s="37"/>
-      <c r="I2" s="40">
+      <c r="I2" s="38">
         <v>1000</v>
       </c>
-      <c r="J2" s="41"/>
-      <c r="K2" s="44">
+      <c r="J2" s="39"/>
+      <c r="K2" s="40">
         <v>10000</v>
       </c>
-      <c r="L2" s="45"/>
-      <c r="M2" s="56">
+      <c r="L2" s="41"/>
+      <c r="M2" s="21">
         <v>20000</v>
       </c>
-      <c r="N2" s="57"/>
-      <c r="O2" s="50">
+      <c r="N2" s="22"/>
+      <c r="O2" s="42">
         <v>100000</v>
       </c>
-      <c r="P2" s="51"/>
-      <c r="Q2" s="54">
+      <c r="P2" s="43"/>
+      <c r="Q2" s="44">
         <v>500000</v>
       </c>
-      <c r="R2" s="55"/>
-      <c r="S2" s="11" t="s">
+      <c r="R2" s="45"/>
+      <c r="S2" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="14">
-        <v>0</v>
-      </c>
-      <c r="D3" s="14">
-        <v>0</v>
-      </c>
-      <c r="E3" s="15">
-        <v>0</v>
-      </c>
-      <c r="F3" s="15">
-        <v>0</v>
-      </c>
-      <c r="G3" s="16">
-        <v>0</v>
-      </c>
-      <c r="H3" s="16">
-        <v>0</v>
-      </c>
-      <c r="I3" s="17">
+      <c r="B3" s="25"/>
+      <c r="C3" s="11">
+        <v>0</v>
+      </c>
+      <c r="D3" s="11">
+        <v>0</v>
+      </c>
+      <c r="E3" s="12">
+        <v>0</v>
+      </c>
+      <c r="F3" s="12">
+        <v>0</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0</v>
+      </c>
+      <c r="H3" s="13">
+        <v>0</v>
+      </c>
+      <c r="I3" s="14">
         <v>1.5169999999999999</v>
       </c>
-      <c r="J3" s="17">
+      <c r="J3" s="14">
         <v>2.0190000000000001</v>
       </c>
-      <c r="K3" s="18">
+      <c r="K3" s="15">
         <v>95.652000000000001</v>
       </c>
-      <c r="L3" s="18">
+      <c r="L3" s="15">
         <v>95.533000000000001</v>
       </c>
-      <c r="M3" s="19">
+      <c r="M3" s="16">
         <v>405.09100000000001</v>
       </c>
-      <c r="N3" s="19">
+      <c r="N3" s="16">
         <v>446.76499999999999</v>
       </c>
-      <c r="O3" s="20">
+      <c r="O3" s="17">
         <v>10283.782999999999</v>
       </c>
-      <c r="P3" s="20">
+      <c r="P3" s="17">
         <v>15858.123</v>
       </c>
-      <c r="Q3" s="58" t="s">
+      <c r="Q3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="59"/>
-      <c r="S3" s="12">
+      <c r="R3" s="24"/>
+      <c r="S3" s="9">
         <f>AVERAGE(C3:R3)</f>
         <v>1942.0345</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="14">
-        <v>0</v>
-      </c>
-      <c r="D4" s="14">
-        <v>0</v>
-      </c>
-      <c r="E4" s="15">
-        <v>0</v>
-      </c>
-      <c r="F4" s="15">
-        <v>0</v>
-      </c>
-      <c r="G4" s="16">
-        <v>0</v>
-      </c>
-      <c r="H4" s="16">
-        <v>0</v>
-      </c>
-      <c r="I4" s="17">
+      <c r="B4" s="25"/>
+      <c r="C4" s="11">
+        <v>0</v>
+      </c>
+      <c r="D4" s="11">
+        <v>0</v>
+      </c>
+      <c r="E4" s="12">
+        <v>0</v>
+      </c>
+      <c r="F4" s="12">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13">
+        <v>0</v>
+      </c>
+      <c r="H4" s="13">
+        <v>0</v>
+      </c>
+      <c r="I4" s="14">
         <v>2.5179999999999998</v>
       </c>
-      <c r="J4" s="17">
+      <c r="J4" s="14">
         <v>3.1059999999999999</v>
       </c>
-      <c r="K4" s="18">
+      <c r="K4" s="15">
         <v>170.49700000000001</v>
       </c>
-      <c r="L4" s="18">
+      <c r="L4" s="15">
         <v>174.483</v>
       </c>
-      <c r="M4" s="19">
+      <c r="M4" s="16">
         <v>736.30600000000004</v>
       </c>
-      <c r="N4" s="19">
+      <c r="N4" s="16">
         <v>787.43700000000001</v>
       </c>
-      <c r="O4" s="20">
+      <c r="O4" s="17">
         <v>13341.522000000001</v>
       </c>
-      <c r="P4" s="20">
+      <c r="P4" s="17">
         <v>14271.179</v>
       </c>
-      <c r="Q4" s="58" t="s">
+      <c r="Q4" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="R4" s="59"/>
-      <c r="S4" s="12">
+      <c r="R4" s="24"/>
+      <c r="S4" s="9">
         <f t="shared" ref="S4:S8" si="0">AVERAGE(C4:R4)</f>
         <v>2106.2177142857145</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="14">
-        <v>0</v>
-      </c>
-      <c r="D5" s="14">
-        <v>0</v>
-      </c>
-      <c r="E5" s="15">
-        <v>0</v>
-      </c>
-      <c r="F5" s="15">
-        <v>0</v>
-      </c>
-      <c r="G5" s="16">
-        <v>0</v>
-      </c>
-      <c r="H5" s="16">
-        <v>0</v>
-      </c>
-      <c r="I5" s="17">
+      <c r="B5" s="25"/>
+      <c r="C5" s="11">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11">
+        <v>0</v>
+      </c>
+      <c r="E5" s="12">
+        <v>0</v>
+      </c>
+      <c r="F5" s="12">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="14">
         <v>7.0359999999999996</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="14">
         <v>14.714</v>
       </c>
-      <c r="K5" s="18">
+      <c r="K5" s="15">
         <v>784.29399999999998</v>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="15">
         <v>726.31399999999996</v>
       </c>
-      <c r="M5" s="19">
+      <c r="M5" s="16">
         <v>3085.8739999999998</v>
       </c>
-      <c r="N5" s="19">
+      <c r="N5" s="16">
         <v>3188.3470000000002</v>
       </c>
-      <c r="O5" s="20">
+      <c r="O5" s="17">
         <v>65010.446000000004</v>
       </c>
-      <c r="P5" s="20">
+      <c r="P5" s="17">
         <v>67090.979000000007</v>
       </c>
-      <c r="Q5" s="58" t="s">
+      <c r="Q5" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="R5" s="59"/>
-      <c r="S5" s="12">
-        <f t="shared" si="0"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="9">
+        <f>AVERAGE(C5:R5)</f>
         <v>9993.4288571428588</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="14">
-        <v>0</v>
-      </c>
-      <c r="D6" s="14">
-        <v>0</v>
-      </c>
-      <c r="E6" s="15">
-        <v>0</v>
-      </c>
-      <c r="F6" s="15">
-        <v>0</v>
-      </c>
-      <c r="G6" s="16">
-        <v>0</v>
-      </c>
-      <c r="H6" s="16">
-        <v>0</v>
-      </c>
-      <c r="I6" s="17">
+      <c r="B6" s="25"/>
+      <c r="C6" s="11">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11">
+        <v>0</v>
+      </c>
+      <c r="E6" s="12">
+        <v>0</v>
+      </c>
+      <c r="F6" s="12">
+        <v>0</v>
+      </c>
+      <c r="G6" s="13">
+        <v>0</v>
+      </c>
+      <c r="H6" s="13">
+        <v>0</v>
+      </c>
+      <c r="I6" s="14">
         <v>1.5169999999999999</v>
       </c>
-      <c r="J6" s="17">
+      <c r="J6" s="14">
         <v>1.002</v>
       </c>
-      <c r="K6" s="18">
+      <c r="K6" s="15">
         <v>5.1230000000000002</v>
       </c>
-      <c r="L6" s="18">
+      <c r="L6" s="15">
         <v>6.6509999999999998</v>
       </c>
-      <c r="M6" s="19">
+      <c r="M6" s="16">
         <v>10.539</v>
       </c>
-      <c r="N6" s="19">
+      <c r="N6" s="16">
         <v>11.895</v>
       </c>
-      <c r="O6" s="20">
+      <c r="O6" s="17">
         <v>65.218000000000004</v>
       </c>
-      <c r="P6" s="20">
+      <c r="P6" s="17">
         <v>86.474000000000004</v>
       </c>
-      <c r="Q6" s="21">
+      <c r="Q6" s="18">
         <v>195.15799999999999</v>
       </c>
-      <c r="R6" s="21">
+      <c r="R6" s="18">
         <v>212.476</v>
       </c>
-      <c r="S6" s="12">
+      <c r="S6" s="9">
         <f t="shared" si="0"/>
         <v>37.2533125</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="14">
-        <v>0</v>
-      </c>
-      <c r="D7" s="14">
-        <v>0</v>
-      </c>
-      <c r="E7" s="15">
-        <v>0</v>
-      </c>
-      <c r="F7" s="15">
-        <v>0</v>
-      </c>
-      <c r="G7" s="16">
-        <v>0</v>
-      </c>
-      <c r="H7" s="16">
-        <v>0</v>
-      </c>
-      <c r="I7" s="17">
+      <c r="B7" s="25"/>
+      <c r="C7" s="11">
+        <v>0</v>
+      </c>
+      <c r="D7" s="11">
+        <v>0</v>
+      </c>
+      <c r="E7" s="12">
+        <v>0</v>
+      </c>
+      <c r="F7" s="12">
+        <v>0</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0</v>
+      </c>
+      <c r="I7" s="14">
         <v>1.5169999999999999</v>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="14">
         <v>1.002</v>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="15">
         <v>5.008</v>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="15">
         <v>3.9910000000000001</v>
       </c>
-      <c r="M7" s="19">
+      <c r="M7" s="16">
         <v>8.43</v>
       </c>
-      <c r="N7" s="19">
+      <c r="N7" s="16">
         <v>10.563000000000001</v>
       </c>
-      <c r="O7" s="20">
+      <c r="O7" s="17">
         <v>55.917000000000002</v>
       </c>
-      <c r="P7" s="20">
+      <c r="P7" s="17">
         <v>70.751999999999995</v>
       </c>
-      <c r="Q7" s="21">
+      <c r="Q7" s="18">
         <v>246.233</v>
       </c>
-      <c r="R7" s="21">
+      <c r="R7" s="18">
         <v>238.62299999999999</v>
       </c>
-      <c r="S7" s="12">
+      <c r="S7" s="9">
         <f t="shared" si="0"/>
         <v>40.127250000000004</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="14">
-        <v>0</v>
-      </c>
-      <c r="D8" s="14">
-        <v>0</v>
-      </c>
-      <c r="E8" s="15">
-        <v>0</v>
-      </c>
-      <c r="F8" s="15">
-        <v>0</v>
-      </c>
-      <c r="G8" s="16">
-        <v>0</v>
-      </c>
-      <c r="H8" s="16">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6">
-        <v>0</v>
-      </c>
-      <c r="K8" s="7">
+      <c r="B8" s="25"/>
+      <c r="C8" s="11">
+        <v>0</v>
+      </c>
+      <c r="D8" s="11">
+        <v>0</v>
+      </c>
+      <c r="E8" s="12">
+        <v>0</v>
+      </c>
+      <c r="F8" s="12">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4">
         <v>2.5259999999999998</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="4">
         <v>0.998</v>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="5">
         <v>4.53</v>
       </c>
-      <c r="N8" s="8">
+      <c r="N8" s="5">
         <v>3.5529999999999999</v>
       </c>
-      <c r="O8" s="9">
+      <c r="O8" s="6">
         <v>17.86</v>
       </c>
-      <c r="P8" s="9">
+      <c r="P8" s="6">
         <v>12.606999999999999</v>
       </c>
-      <c r="Q8" s="10">
+      <c r="Q8" s="7">
         <v>77.991</v>
       </c>
-      <c r="R8" s="10">
+      <c r="R8" s="7">
         <v>76.984999999999999</v>
       </c>
-      <c r="S8" s="12">
+      <c r="S8" s="9">
         <f t="shared" si="0"/>
         <v>12.315625000000001</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29" t="s">
+      <c r="D9" s="20"/>
+      <c r="E9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29" t="s">
+      <c r="F9" s="20"/>
+      <c r="G9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29" t="s">
+      <c r="H9" s="20"/>
+      <c r="I9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="29"/>
-      <c r="K9" s="29" t="s">
+      <c r="J9" s="20"/>
+      <c r="K9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="L9" s="29"/>
-      <c r="M9" s="29" t="s">
+      <c r="L9" s="20"/>
+      <c r="M9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N9" s="29"/>
-      <c r="O9" s="29" t="s">
+      <c r="N9" s="20"/>
+      <c r="O9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="29" t="s">
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="R9" s="29"/>
+      <c r="R9" s="20"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
@@ -1740,23 +1845,7 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="K1:L1"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="O1:P1"/>
@@ -1773,7 +1862,23 @@
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="M9:N9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
Se realizan mas pruebas y por ende el único archivo alterado es el .xlsx
</commit_message>
<xml_diff>
--- a/Tarea#2.xlsx
+++ b/Tarea#2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unitechn-my.sharepoint.com/personal/ema_castellanos_unitec_edu/Documents/2026/Q2 2026/analisis de algoritmos/Semana 6/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="209" documentId="8_{EBE05390-39BD-48B3-B14E-C882FAC2D8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B87DC15-EDB2-4388-8534-3942377A771A}"/>
+  <xr:revisionPtr revIDLastSave="264" documentId="8_{EBE05390-39BD-48B3-B14E-C882FAC2D8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8640181-37D7-4B11-A073-76FC38E72660}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{0331FB16-A420-4772-893E-678055F07C6C}"/>
   </bookViews>
@@ -40,6 +40,60 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={EC783D3F-A939-4FF4-B399-EA1C036939F2}</author>
+    <author>tc={71CAF469-6971-48AB-8836-FE597D51049A}</author>
+    <author>tc={CC83B886-9E33-4467-AF5C-30AC00687B06}</author>
+    <author>tc={A992F360-4CA1-4D8A-92B0-9F2374F4D4B3}</author>
+    <author>tc={9F51FF6E-3D9F-4E46-8E79-2B8E3D46C532}</author>
+  </authors>
+  <commentList>
+    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{EC783D3F-A939-4FF4-B399-EA1C036939F2}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Error provocado por el insertion sort durante ejecución</t>
+      </text>
+    </comment>
+    <comment ref="P3" authorId="1" shapeId="0" xr:uid="{71CAF469-6971-48AB-8836-FE597D51049A}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Se comenta en prueba 7.2 por problema en 7.a</t>
+      </text>
+    </comment>
+    <comment ref="O6" authorId="2" shapeId="0" xr:uid="{CC83B886-9E33-4467-AF5C-30AC00687B06}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Error provocado por el insertion sort</t>
+      </text>
+    </comment>
+    <comment ref="O7" authorId="3" shapeId="0" xr:uid="{A992F360-4CA1-4D8A-92B0-9F2374F4D4B3}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Error provocado por el insertion sort durante ejecución</t>
+      </text>
+    </comment>
+    <comment ref="O8" authorId="4" shapeId="0" xr:uid="{9F51FF6E-3D9F-4E46-8E79-2B8E3D46C532}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    Error provocado por el insertion sort durante ejecución</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={079B16CC-2696-4C04-835E-03E2061C0AD6}</author>
@@ -76,23 +130,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="22">
   <si>
     <t>Algoritmo</t>
   </si>
   <si>
-    <t>Prueba 1 (s)</t>
-  </si>
-  <si>
-    <t>Prueba 2 (s)</t>
-  </si>
-  <si>
-    <t>Prueba 3 (s)</t>
-  </si>
-  <si>
-    <t>Promedio (s)</t>
-  </si>
-  <si>
     <t>Insertion Sort</t>
   </si>
   <si>
@@ -100,21 +142,6 @@
   </si>
   <si>
     <t>Cantidad de elementos</t>
-  </si>
-  <si>
-    <t>Prueba 4 (s)</t>
-  </si>
-  <si>
-    <t>Prueba 5 (s)</t>
-  </si>
-  <si>
-    <t>Prueba 6 (s)</t>
-  </si>
-  <si>
-    <t>Prueba 7 (s)</t>
-  </si>
-  <si>
-    <t>Prueba 8 (s)</t>
   </si>
   <si>
     <t>n/a</t>
@@ -179,7 +206,7 @@
     <numFmt numFmtId="164" formatCode="0.00000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,6 +239,12 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -378,7 +411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -433,9 +466,6 @@
     </xf>
     <xf numFmtId="165" fontId="1" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -888,6 +918,26 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="O3" dT="2026-05-30T14:07:25.82" personId="{295C8FAE-595D-49B2-B473-4AB46D987526}" id="{EC783D3F-A939-4FF4-B399-EA1C036939F2}">
+    <text>Error provocado por el insertion sort durante ejecución</text>
+  </threadedComment>
+  <threadedComment ref="P3" dT="2026-05-30T14:12:04.75" personId="{295C8FAE-595D-49B2-B473-4AB46D987526}" id="{71CAF469-6971-48AB-8836-FE597D51049A}">
+    <text>Se comenta en prueba 7.2 por problema en 7.a</text>
+  </threadedComment>
+  <threadedComment ref="O6" dT="2026-05-30T14:07:25.82" personId="{295C8FAE-595D-49B2-B473-4AB46D987526}" id="{CC83B886-9E33-4467-AF5C-30AC00687B06}">
+    <text>Error provocado por el insertion sort</text>
+  </threadedComment>
+  <threadedComment ref="O7" dT="2026-05-30T14:07:25.82" personId="{295C8FAE-595D-49B2-B473-4AB46D987526}" id="{A992F360-4CA1-4D8A-92B0-9F2374F4D4B3}">
+    <text>Error provocado por el insertion sort durante ejecución</text>
+  </threadedComment>
+  <threadedComment ref="O8" dT="2026-05-30T14:07:25.82" personId="{295C8FAE-595D-49B2-B473-4AB46D987526}" id="{9F51FF6E-3D9F-4E46-8E79-2B8E3D46C532}">
+    <text>Error provocado por el insertion sort durante ejecución</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="Q3" dT="2026-05-30T04:46:31.55" personId="{295C8FAE-595D-49B2-B473-4AB46D987526}" id="{079B16CC-2696-4C04-835E-03E2061C0AD6}">
     <text>Pasaron 20 minutos y nada</text>
   </threadedComment>
@@ -901,106 +951,104 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9833A91-1209-464F-8079-D46E86F49EA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9833A91-1209-464F-8079-D46E86F49EA6}">
   <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.88671875" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="17" width="15.6640625" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" customWidth="1"/>
-    <col min="19" max="19" width="15.44140625" style="10" customWidth="1"/>
+    <col min="18" max="18" width="16.109375" customWidth="1"/>
+    <col min="19" max="19" width="17.6640625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="47" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="48"/>
-      <c r="E1" s="49" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="50"/>
-      <c r="G1" s="51" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="52"/>
-      <c r="I1" s="53" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="54"/>
-      <c r="K1" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="56"/>
-      <c r="M1" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="27"/>
-      <c r="O1" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="R1" s="31"/>
+      <c r="C1" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="47"/>
+      <c r="E1" s="48" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="49"/>
+      <c r="G1" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="51"/>
+      <c r="I1" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="53"/>
+      <c r="K1" s="54" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="55"/>
+      <c r="M1" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="26"/>
+      <c r="O1" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="30"/>
       <c r="S1" s="8" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="46"/>
+      <c r="A2" s="45"/>
       <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="32">
+        <v>3</v>
+      </c>
+      <c r="C2" s="31">
         <v>5</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="34">
+      <c r="D2" s="32"/>
+      <c r="E2" s="33">
         <v>10</v>
       </c>
-      <c r="F2" s="35"/>
-      <c r="G2" s="36">
+      <c r="F2" s="34"/>
+      <c r="G2" s="35">
         <v>100</v>
       </c>
-      <c r="H2" s="37"/>
-      <c r="I2" s="38">
+      <c r="H2" s="36"/>
+      <c r="I2" s="37">
         <v>1000</v>
       </c>
-      <c r="J2" s="39"/>
-      <c r="K2" s="40">
+      <c r="J2" s="38"/>
+      <c r="K2" s="39">
         <v>5000</v>
       </c>
-      <c r="L2" s="41"/>
-      <c r="M2" s="19">
+      <c r="L2" s="40"/>
+      <c r="M2" s="20">
         <v>10000</v>
       </c>
-      <c r="N2" s="19">
-        <v>10000</v>
-      </c>
-      <c r="O2" s="42">
+      <c r="N2" s="21"/>
+      <c r="O2" s="41">
         <v>100000</v>
       </c>
-      <c r="P2" s="43"/>
-      <c r="Q2" s="44">
+      <c r="P2" s="42"/>
+      <c r="Q2" s="43">
         <v>500000</v>
       </c>
-      <c r="R2" s="45"/>
+      <c r="R2" s="44"/>
       <c r="S2" s="8" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="25"/>
+      <c r="A3" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24"/>
       <c r="C3" s="11">
         <v>0</v>
       </c>
@@ -1025,8 +1073,12 @@
       <c r="J3" s="14">
         <v>3.01</v>
       </c>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+      <c r="K3" s="15">
+        <v>25.021999999999998</v>
+      </c>
+      <c r="L3" s="15">
+        <v>89.974999999999994</v>
+      </c>
       <c r="M3" s="16">
         <v>177.99799999999999</v>
       </c>
@@ -1034,27 +1086,27 @@
         <v>113.999</v>
       </c>
       <c r="O3" s="17" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="P3" s="17" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="S3" s="9">
         <f>AVERAGE(C3:R3)</f>
-        <v>29.601299999999998</v>
+        <v>34.250833333333333</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="25"/>
+      <c r="A4" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="24"/>
       <c r="C4" s="11">
         <v>0</v>
       </c>
@@ -1079,36 +1131,40 @@
       <c r="J4" s="14">
         <v>5.9969999999999999</v>
       </c>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
+      <c r="K4" s="15">
+        <v>106.003</v>
+      </c>
+      <c r="L4" s="15">
+        <v>105.01600000000001</v>
+      </c>
       <c r="M4" s="16">
         <v>878.59400000000005</v>
       </c>
       <c r="N4" s="16">
         <v>472.16699999999997</v>
       </c>
-      <c r="O4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="P4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q4" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="R4" s="18" t="s">
-        <v>19</v>
+      <c r="O4" s="17">
+        <v>41228.805</v>
+      </c>
+      <c r="P4" s="17">
+        <v>40505.779000000002</v>
+      </c>
+      <c r="Q4" s="18">
+        <v>545093.53500000003</v>
+      </c>
+      <c r="R4" s="18">
+        <v>382173.02</v>
       </c>
       <c r="S4" s="9">
         <f t="shared" ref="S4:S8" si="0">AVERAGE(C4:R4)</f>
-        <v>136.07689999999999</v>
+        <v>63160.807937500002</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="25"/>
+      <c r="A5" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="24"/>
       <c r="C5" s="11">
         <v>0</v>
       </c>
@@ -1133,36 +1189,40 @@
       <c r="J5" s="14">
         <v>7.9930000000000003</v>
       </c>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
+      <c r="K5" s="15">
+        <v>198.00899999999999</v>
+      </c>
+      <c r="L5" s="15">
+        <v>191.012</v>
+      </c>
       <c r="M5" s="16">
         <v>1019.189</v>
       </c>
       <c r="N5" s="16">
         <v>973.73699999999997</v>
       </c>
-      <c r="O5" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="P5" s="17" t="s">
-        <v>18</v>
+      <c r="O5" s="17">
+        <v>86683.131999999998</v>
+      </c>
+      <c r="P5" s="17">
+        <v>88365.824999999997</v>
       </c>
       <c r="Q5" s="18" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="R5" s="18" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="S5" s="9">
         <f t="shared" si="0"/>
-        <v>201.19380000000001</v>
+        <v>12674.994000000001</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="25"/>
+      <c r="A6" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="24"/>
       <c r="C6" s="11">
         <v>0</v>
       </c>
@@ -1187,28 +1247,40 @@
       <c r="J6" s="14">
         <v>2.0009999999999999</v>
       </c>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
+      <c r="K6" s="15">
+        <v>3.99</v>
+      </c>
+      <c r="L6" s="15">
+        <v>3.99</v>
+      </c>
       <c r="M6" s="16">
         <v>56.994999999999997</v>
       </c>
       <c r="N6" s="16">
         <v>6.992</v>
       </c>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
+      <c r="O6" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="P6" s="17">
+        <v>69.006</v>
+      </c>
+      <c r="Q6" s="18">
+        <v>213.13499999999999</v>
+      </c>
+      <c r="R6" s="18">
+        <v>200.023</v>
+      </c>
       <c r="S6" s="9">
         <f t="shared" si="0"/>
-        <v>6.5987999999999998</v>
+        <v>37.075466666666664</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="25"/>
+      <c r="A7" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="24"/>
       <c r="C7" s="11">
         <v>0</v>
       </c>
@@ -1233,28 +1305,40 @@
       <c r="J7" s="14">
         <v>0</v>
       </c>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
+      <c r="K7" s="15">
+        <v>2.0059999999999998</v>
+      </c>
+      <c r="L7" s="15">
+        <v>1.99</v>
+      </c>
       <c r="M7" s="16">
         <v>7.9960000000000004</v>
       </c>
       <c r="N7" s="16">
         <v>3.9929999999999999</v>
       </c>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
+      <c r="O7" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="P7" s="17">
+        <v>56.558999999999997</v>
+      </c>
+      <c r="Q7" s="18">
+        <v>243.58799999999999</v>
+      </c>
+      <c r="R7" s="18">
+        <v>216.43199999999999</v>
+      </c>
       <c r="S7" s="9">
         <f t="shared" si="0"/>
-        <v>1.1989000000000001</v>
+        <v>35.504266666666666</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="25"/>
+      <c r="A8" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="24"/>
       <c r="C8" s="11">
         <v>0</v>
       </c>
@@ -1279,59 +1363,71 @@
       <c r="J8" s="3">
         <v>0</v>
       </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="K8" s="4">
+        <v>1.9910000000000001</v>
+      </c>
+      <c r="L8" s="4">
+        <v>7.0039999999999996</v>
+      </c>
       <c r="M8" s="5">
         <v>6.98</v>
       </c>
       <c r="N8" s="5">
         <v>2.9980000000000002</v>
       </c>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
+      <c r="O8" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="P8" s="6">
+        <v>34.552</v>
+      </c>
+      <c r="Q8" s="7">
+        <v>129.19300000000001</v>
+      </c>
+      <c r="R8" s="7">
+        <v>138.773</v>
+      </c>
       <c r="S8" s="9">
         <f t="shared" si="0"/>
-        <v>0.99780000000000013</v>
+        <v>21.432733333333331</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="L9" s="20"/>
-      <c r="M9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="R9" s="20"/>
+      <c r="C9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="R9" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C9:D9"/>
@@ -1357,6 +1453,7 @@
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
     <mergeCell ref="Q1:R1"/>
     <mergeCell ref="Q2:R2"/>
     <mergeCell ref="O9:P9"/>
@@ -1365,6 +1462,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1381,92 +1479,92 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="48"/>
-      <c r="E1" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="50"/>
-      <c r="G1" s="51" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="52"/>
-      <c r="I1" s="53" t="s">
-        <v>25</v>
-      </c>
-      <c r="J1" s="54"/>
-      <c r="K1" s="55" t="s">
-        <v>26</v>
-      </c>
-      <c r="L1" s="56"/>
-      <c r="M1" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="27"/>
-      <c r="O1" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="R1" s="31"/>
+      <c r="C1" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="47"/>
+      <c r="E1" s="48" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="49"/>
+      <c r="G1" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="51"/>
+      <c r="I1" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="53"/>
+      <c r="K1" s="54" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="55"/>
+      <c r="M1" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="26"/>
+      <c r="O1" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="30"/>
       <c r="S1" s="8" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="46"/>
+      <c r="A2" s="45"/>
       <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="32">
+        <v>3</v>
+      </c>
+      <c r="C2" s="31">
         <v>5</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="34">
+      <c r="D2" s="32"/>
+      <c r="E2" s="33">
         <v>10</v>
       </c>
-      <c r="F2" s="35"/>
-      <c r="G2" s="36">
+      <c r="F2" s="34"/>
+      <c r="G2" s="35">
         <v>100</v>
       </c>
-      <c r="H2" s="37"/>
-      <c r="I2" s="38">
+      <c r="H2" s="36"/>
+      <c r="I2" s="37">
         <v>1000</v>
       </c>
-      <c r="J2" s="39"/>
-      <c r="K2" s="40">
+      <c r="J2" s="38"/>
+      <c r="K2" s="39">
         <v>10000</v>
       </c>
-      <c r="L2" s="41"/>
-      <c r="M2" s="21">
+      <c r="L2" s="40"/>
+      <c r="M2" s="20">
         <v>20000</v>
       </c>
-      <c r="N2" s="22"/>
-      <c r="O2" s="42">
+      <c r="N2" s="21"/>
+      <c r="O2" s="41">
         <v>100000</v>
       </c>
-      <c r="P2" s="43"/>
-      <c r="Q2" s="44">
+      <c r="P2" s="42"/>
+      <c r="Q2" s="43">
         <v>500000</v>
       </c>
-      <c r="R2" s="45"/>
+      <c r="R2" s="44"/>
       <c r="S2" s="8" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="25"/>
+      <c r="A3" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24"/>
       <c r="C3" s="11">
         <v>0</v>
       </c>
@@ -1509,20 +1607,20 @@
       <c r="P3" s="17">
         <v>15858.123</v>
       </c>
-      <c r="Q3" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="R3" s="24"/>
+      <c r="Q3" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="R3" s="23"/>
       <c r="S3" s="9">
         <f>AVERAGE(C3:R3)</f>
         <v>1942.0345</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="25"/>
+      <c r="A4" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="24"/>
       <c r="C4" s="11">
         <v>0</v>
       </c>
@@ -1565,20 +1663,20 @@
       <c r="P4" s="17">
         <v>14271.179</v>
       </c>
-      <c r="Q4" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="R4" s="24"/>
+      <c r="Q4" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="R4" s="23"/>
       <c r="S4" s="9">
         <f t="shared" ref="S4:S8" si="0">AVERAGE(C4:R4)</f>
         <v>2106.2177142857145</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="25"/>
+      <c r="A5" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="24"/>
       <c r="C5" s="11">
         <v>0</v>
       </c>
@@ -1621,20 +1719,20 @@
       <c r="P5" s="17">
         <v>67090.979000000007</v>
       </c>
-      <c r="Q5" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="R5" s="24"/>
+      <c r="Q5" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="R5" s="23"/>
       <c r="S5" s="9">
         <f>AVERAGE(C5:R5)</f>
         <v>9993.4288571428588</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="25"/>
+      <c r="A6" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="24"/>
       <c r="C6" s="11">
         <v>0</v>
       </c>
@@ -1689,10 +1787,10 @@
       </c>
     </row>
     <row r="7" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="25"/>
+      <c r="A7" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="24"/>
       <c r="C7" s="11">
         <v>0</v>
       </c>
@@ -1747,10 +1845,10 @@
       </c>
     </row>
     <row r="8" spans="1:19" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="25"/>
+      <c r="A8" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="24"/>
       <c r="C8" s="11">
         <v>0</v>
       </c>
@@ -1805,42 +1903,42 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="L9" s="20"/>
-      <c r="M9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="R9" s="20"/>
+      <c r="C9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="R9" s="19"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>